<commit_message>
feat: sub-group nodes by resource-group field with named boxes
</commit_message>
<xml_diff>
--- a/ourresult/sample.xlsx
+++ b/ourresult/sample.xlsx
@@ -3290,7 +3290,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -4340,7 +4340,7 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr">
@@ -5548,7 +5548,7 @@
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr">
@@ -5598,7 +5598,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="G105" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H111" s="4" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H113" s="4" t="inlineStr">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H117" s="4" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H119" s="4" t="inlineStr">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="G123" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H123" s="4" t="inlineStr">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="G125" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H125" s="4" t="inlineStr">
@@ -6806,7 +6806,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="G129" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H129" s="4" t="inlineStr">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="G131" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H131" s="4" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="G135" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H135" s="4" t="inlineStr">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="G137" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H137" s="4" t="inlineStr">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="G141" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H141" s="4" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="G143" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H143" s="4" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="G147" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H147" s="4" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="G149" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H149" s="4" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="G153" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H153" s="4" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="G155" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H155" s="4" t="inlineStr">
@@ -8322,7 +8322,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="G159" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H159" s="4" t="inlineStr">
@@ -8572,7 +8572,7 @@
       </c>
       <c r="G161" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H161" s="4" t="inlineStr">
@@ -8622,7 +8622,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H164" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="G165" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H165" s="4" t="inlineStr">
@@ -8872,7 +8872,7 @@
       </c>
       <c r="G167" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H167" s="4" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
@@ -9072,7 +9072,7 @@
       </c>
       <c r="G171" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H171" s="4" t="inlineStr">
@@ -9172,7 +9172,7 @@
       </c>
       <c r="G173" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H173" s="4" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
@@ -9372,7 +9372,7 @@
       </c>
       <c r="G177" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H177" s="4" t="inlineStr">
@@ -9472,7 +9472,7 @@
       </c>
       <c r="G179" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H179" s="4" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H182" s="2" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="G183" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H183" s="4" t="inlineStr">
@@ -9780,7 +9780,7 @@
       </c>
       <c r="G185" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H185" s="4" t="inlineStr">
@@ -9830,7 +9830,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
@@ -13380,7 +13380,7 @@
       </c>
       <c r="G257" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H257" s="4" t="inlineStr">
@@ -13430,7 +13430,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
@@ -13530,7 +13530,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr">
@@ -13580,7 +13580,7 @@
       </c>
       <c r="G261" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H261" s="4" t="inlineStr">
@@ -13680,7 +13680,7 @@
       </c>
       <c r="G263" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H263" s="4" t="inlineStr">
@@ -13730,7 +13730,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
@@ -13880,7 +13880,7 @@
       </c>
       <c r="G267" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H267" s="4" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="G269" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H269" s="4" t="inlineStr">
@@ -14030,7 +14030,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr">
@@ -14130,7 +14130,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr">
@@ -14180,7 +14180,7 @@
       </c>
       <c r="G273" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H273" s="4" t="inlineStr">
@@ -14280,7 +14280,7 @@
       </c>
       <c r="G275" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr">
@@ -14330,7 +14330,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr">
@@ -14430,7 +14430,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="G279" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H279" s="4" t="inlineStr">
@@ -14580,7 +14580,7 @@
       </c>
       <c r="G281" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr">
@@ -14638,7 +14638,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
@@ -14738,7 +14738,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">
@@ -14788,7 +14788,7 @@
       </c>
       <c r="G285" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
@@ -14888,7 +14888,7 @@
       </c>
       <c r="G287" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
@@ -14938,7 +14938,7 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
@@ -15038,7 +15038,7 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
@@ -15088,7 +15088,7 @@
       </c>
       <c r="G291" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H291" s="4" t="inlineStr">
@@ -15188,7 +15188,7 @@
       </c>
       <c r="G293" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="G297" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H297" s="4" t="inlineStr">
@@ -15488,7 +15488,7 @@
       </c>
       <c r="G299" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr">
@@ -15538,7 +15538,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -15638,7 +15638,7 @@
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H302" s="2" t="inlineStr">
@@ -15688,7 +15688,7 @@
       </c>
       <c r="G303" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H303" s="4" t="inlineStr">
@@ -15788,7 +15788,7 @@
       </c>
       <c r="G305" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H305" s="4" t="inlineStr">
@@ -15838,7 +15838,7 @@
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H306" s="2" t="inlineStr">
@@ -15946,7 +15946,7 @@
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H308" s="2" t="inlineStr">
@@ -15996,7 +15996,7 @@
       </c>
       <c r="G309" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H309" s="4" t="inlineStr">
@@ -16096,7 +16096,7 @@
       </c>
       <c r="G311" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H311" s="4" t="inlineStr">
@@ -16146,7 +16146,7 @@
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H312" s="2" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H314" s="2" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="G315" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H315" s="4" t="inlineStr">
@@ -16396,7 +16396,7 @@
       </c>
       <c r="G317" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H317" s="4" t="inlineStr">
@@ -16446,7 +16446,7 @@
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H318" s="2" t="inlineStr">
@@ -16546,7 +16546,7 @@
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H320" s="2" t="inlineStr">
@@ -16596,7 +16596,7 @@
       </c>
       <c r="G321" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H321" s="4" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="G323" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H323" s="4" t="inlineStr">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H324" s="2" t="inlineStr">
@@ -16846,7 +16846,7 @@
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H326" s="2" t="inlineStr">
@@ -16896,7 +16896,7 @@
       </c>
       <c r="G327" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H327" s="4" t="inlineStr">
@@ -16996,7 +16996,7 @@
       </c>
       <c r="G329" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H329" s="4" t="inlineStr">
@@ -17046,7 +17046,7 @@
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H330" s="2" t="inlineStr">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H332" s="2" t="inlineStr">
@@ -17204,7 +17204,7 @@
       </c>
       <c r="G333" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H333" s="4" t="inlineStr">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="G335" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H335" s="4" t="inlineStr">
@@ -17354,7 +17354,7 @@
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H336" s="2" t="inlineStr">
@@ -17454,7 +17454,7 @@
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H338" s="2" t="inlineStr">
@@ -17504,7 +17504,7 @@
       </c>
       <c r="G339" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H339" s="4" t="inlineStr">
@@ -17604,7 +17604,7 @@
       </c>
       <c r="G341" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H341" s="4" t="inlineStr">
@@ -17654,7 +17654,7 @@
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H342" s="2" t="inlineStr">
@@ -17754,7 +17754,7 @@
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H344" s="2" t="inlineStr">
@@ -17804,7 +17804,7 @@
       </c>
       <c r="G345" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H345" s="4" t="inlineStr">
@@ -17904,7 +17904,7 @@
       </c>
       <c r="G347" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H347" s="4" t="inlineStr">
@@ -17954,7 +17954,7 @@
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H348" s="2" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H350" s="2" t="inlineStr">
@@ -18104,7 +18104,7 @@
       </c>
       <c r="G351" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H351" s="4" t="inlineStr">
@@ -18204,7 +18204,7 @@
       </c>
       <c r="G353" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H353" s="4" t="inlineStr">
@@ -18254,7 +18254,7 @@
       </c>
       <c r="G354" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H354" s="2" t="inlineStr">
@@ -18354,7 +18354,7 @@
       </c>
       <c r="G356" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H356" s="2" t="inlineStr">
@@ -18412,7 +18412,7 @@
       </c>
       <c r="G357" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H357" s="4" t="inlineStr">
@@ -18512,7 +18512,7 @@
       </c>
       <c r="G359" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H359" s="4" t="inlineStr">
@@ -18562,7 +18562,7 @@
       </c>
       <c r="G360" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H360" s="2" t="inlineStr">
@@ -18662,7 +18662,7 @@
       </c>
       <c r="G362" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H362" s="2" t="inlineStr">
@@ -18712,7 +18712,7 @@
       </c>
       <c r="G363" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H363" s="4" t="inlineStr">
@@ -18812,7 +18812,7 @@
       </c>
       <c r="G365" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H365" s="4" t="inlineStr">
@@ -18862,7 +18862,7 @@
       </c>
       <c r="G366" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H366" s="2" t="inlineStr">
@@ -18962,7 +18962,7 @@
       </c>
       <c r="G368" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H368" s="2" t="inlineStr">
@@ -19012,7 +19012,7 @@
       </c>
       <c r="G369" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H369" s="4" t="inlineStr">
@@ -19112,7 +19112,7 @@
       </c>
       <c r="G371" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H371" s="4" t="inlineStr">
@@ -19162,7 +19162,7 @@
       </c>
       <c r="G372" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H372" s="2" t="inlineStr">
@@ -19262,7 +19262,7 @@
       </c>
       <c r="G374" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H374" s="2" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="G375" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H375" s="4" t="inlineStr">
@@ -19412,7 +19412,7 @@
       </c>
       <c r="G377" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H377" s="4" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H378" s="2" t="inlineStr">
@@ -19562,7 +19562,7 @@
       </c>
       <c r="G380" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H380" s="2" t="inlineStr">
@@ -19612,7 +19612,7 @@
       </c>
       <c r="G381" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H381" s="4" t="inlineStr">
@@ -19720,7 +19720,7 @@
       </c>
       <c r="G383" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H383" s="4" t="inlineStr">
@@ -19770,7 +19770,7 @@
       </c>
       <c r="G384" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H384" s="2" t="inlineStr">
@@ -19870,7 +19870,7 @@
       </c>
       <c r="G386" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H386" s="2" t="inlineStr">
@@ -19920,7 +19920,7 @@
       </c>
       <c r="G387" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H387" s="4" t="inlineStr">
@@ -23470,7 +23470,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="G459" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H459" s="4" t="inlineStr">
@@ -23620,7 +23620,7 @@
       </c>
       <c r="G461" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H461" s="4" t="inlineStr">
@@ -23670,7 +23670,7 @@
       </c>
       <c r="G462" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H462" s="2" t="inlineStr">
@@ -23770,7 +23770,7 @@
       </c>
       <c r="G464" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H464" s="2" t="inlineStr">
@@ -23820,7 +23820,7 @@
       </c>
       <c r="G465" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H465" s="4" t="inlineStr">
@@ -23920,7 +23920,7 @@
       </c>
       <c r="G467" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H467" s="4" t="inlineStr">
@@ -23970,7 +23970,7 @@
       </c>
       <c r="G468" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H468" s="2" t="inlineStr">
@@ -24070,7 +24070,7 @@
       </c>
       <c r="G470" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H470" s="2" t="inlineStr">
@@ -24120,7 +24120,7 @@
       </c>
       <c r="G471" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H471" s="4" t="inlineStr">
@@ -24220,7 +24220,7 @@
       </c>
       <c r="G473" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H473" s="4" t="inlineStr">
@@ -24270,7 +24270,7 @@
       </c>
       <c r="G474" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H474" s="2" t="inlineStr">
@@ -24370,7 +24370,7 @@
       </c>
       <c r="G476" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H476" s="2" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="G477" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H477" s="4" t="inlineStr">
@@ -24520,7 +24520,7 @@
       </c>
       <c r="G479" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H479" s="4" t="inlineStr">
@@ -24570,7 +24570,7 @@
       </c>
       <c r="G480" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H480" s="2" t="inlineStr">
@@ -24670,7 +24670,7 @@
       </c>
       <c r="G482" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H482" s="2" t="inlineStr">
@@ -24728,7 +24728,7 @@
       </c>
       <c r="G483" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H483" s="4" t="inlineStr">
@@ -24828,7 +24828,7 @@
       </c>
       <c r="G485" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H485" s="4" t="inlineStr">
@@ -24878,7 +24878,7 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
@@ -24978,7 +24978,7 @@
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
@@ -25028,7 +25028,7 @@
       </c>
       <c r="G489" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H489" s="4" t="inlineStr">
@@ -25128,7 +25128,7 @@
       </c>
       <c r="G491" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H491" s="4" t="inlineStr">
@@ -25178,7 +25178,7 @@
       </c>
       <c r="G492" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H492" s="2" t="inlineStr">
@@ -25278,7 +25278,7 @@
       </c>
       <c r="G494" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H494" s="2" t="inlineStr">
@@ -25328,7 +25328,7 @@
       </c>
       <c r="G495" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H495" s="4" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="G497" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H497" s="4" t="inlineStr">
@@ -25478,7 +25478,7 @@
       </c>
       <c r="G498" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H498" s="2" t="inlineStr">
@@ -25578,7 +25578,7 @@
       </c>
       <c r="G500" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H500" s="2" t="inlineStr">
@@ -25628,7 +25628,7 @@
       </c>
       <c r="G501" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H501" s="4" t="inlineStr">
@@ -25728,7 +25728,7 @@
       </c>
       <c r="G503" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H503" s="4" t="inlineStr">
@@ -25778,7 +25778,7 @@
       </c>
       <c r="G504" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H504" s="2" t="inlineStr">
@@ -25878,7 +25878,7 @@
       </c>
       <c r="G506" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H506" s="2" t="inlineStr">
@@ -25928,7 +25928,7 @@
       </c>
       <c r="G507" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H507" s="4" t="inlineStr">
@@ -26036,7 +26036,7 @@
       </c>
       <c r="G509" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H509" s="4" t="inlineStr">
@@ -26086,7 +26086,7 @@
       </c>
       <c r="G510" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H510" s="2" t="inlineStr">
@@ -26186,7 +26186,7 @@
       </c>
       <c r="G512" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H512" s="2" t="inlineStr">
@@ -26236,7 +26236,7 @@
       </c>
       <c r="G513" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H513" s="4" t="inlineStr">
@@ -26336,7 +26336,7 @@
       </c>
       <c r="G515" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H515" s="4" t="inlineStr">
@@ -26386,7 +26386,7 @@
       </c>
       <c r="G516" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H516" s="2" t="inlineStr">
@@ -26486,7 +26486,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -26536,7 +26536,7 @@
       </c>
       <c r="G519" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H519" s="4" t="inlineStr">
@@ -26636,7 +26636,7 @@
       </c>
       <c r="G521" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H521" s="4" t="inlineStr">
@@ -26686,7 +26686,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -26786,7 +26786,7 @@
       </c>
       <c r="G524" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H524" s="2" t="inlineStr">
@@ -26836,7 +26836,7 @@
       </c>
       <c r="G525" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H525" s="4" t="inlineStr">
@@ -26936,7 +26936,7 @@
       </c>
       <c r="G527" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H527" s="4" t="inlineStr">
@@ -26986,7 +26986,7 @@
       </c>
       <c r="G528" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H528" s="2" t="inlineStr">
@@ -27086,7 +27086,7 @@
       </c>
       <c r="G530" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H530" s="2" t="inlineStr">
@@ -27136,7 +27136,7 @@
       </c>
       <c r="G531" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H531" s="4" t="inlineStr">
@@ -27244,7 +27244,7 @@
       </c>
       <c r="G533" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H533" s="4" t="inlineStr">
@@ -27294,7 +27294,7 @@
       </c>
       <c r="G534" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H534" s="2" t="inlineStr">
@@ -27394,7 +27394,7 @@
       </c>
       <c r="G536" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H536" s="2" t="inlineStr">
@@ -27444,7 +27444,7 @@
       </c>
       <c r="G537" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H537" s="4" t="inlineStr">
@@ -27544,7 +27544,7 @@
       </c>
       <c r="G539" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H539" s="4" t="inlineStr">
@@ -27594,7 +27594,7 @@
       </c>
       <c r="G540" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H540" s="2" t="inlineStr">
@@ -27694,7 +27694,7 @@
       </c>
       <c r="G542" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H542" s="2" t="inlineStr">
@@ -27744,7 +27744,7 @@
       </c>
       <c r="G543" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H543" s="4" t="inlineStr">
@@ -27844,7 +27844,7 @@
       </c>
       <c r="G545" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H545" s="4" t="inlineStr">
@@ -27894,7 +27894,7 @@
       </c>
       <c r="G546" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H546" s="2" t="inlineStr">
@@ -27994,7 +27994,7 @@
       </c>
       <c r="G548" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H548" s="2" t="inlineStr">
@@ -28044,7 +28044,7 @@
       </c>
       <c r="G549" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H549" s="4" t="inlineStr">
@@ -28144,7 +28144,7 @@
       </c>
       <c r="G551" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H551" s="4" t="inlineStr">
@@ -28194,7 +28194,7 @@
       </c>
       <c r="G552" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H552" s="2" t="inlineStr">
@@ -28294,7 +28294,7 @@
       </c>
       <c r="G554" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H554" s="2" t="inlineStr">
@@ -28344,7 +28344,7 @@
       </c>
       <c r="G555" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H555" s="4" t="inlineStr">
@@ -28444,7 +28444,7 @@
       </c>
       <c r="G557" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H557" s="4" t="inlineStr">
@@ -28502,7 +28502,7 @@
       </c>
       <c r="G558" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H558" s="2" t="inlineStr">
@@ -28602,7 +28602,7 @@
       </c>
       <c r="G560" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H560" s="2" t="inlineStr">
@@ -28652,7 +28652,7 @@
       </c>
       <c r="G561" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H561" s="4" t="inlineStr">
@@ -28752,7 +28752,7 @@
       </c>
       <c r="G563" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H563" s="4" t="inlineStr">
@@ -28802,7 +28802,7 @@
       </c>
       <c r="G564" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H564" s="2" t="inlineStr">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="G566" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H566" s="2" t="inlineStr">
@@ -28952,7 +28952,7 @@
       </c>
       <c r="G567" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H567" s="4" t="inlineStr">
@@ -29052,7 +29052,7 @@
       </c>
       <c r="G569" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H569" s="4" t="inlineStr">
@@ -29102,7 +29102,7 @@
       </c>
       <c r="G570" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H570" s="2" t="inlineStr">
@@ -29202,7 +29202,7 @@
       </c>
       <c r="G572" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H572" s="2" t="inlineStr">
@@ -29252,7 +29252,7 @@
       </c>
       <c r="G573" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H573" s="4" t="inlineStr">
@@ -29352,7 +29352,7 @@
       </c>
       <c r="G575" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H575" s="4" t="inlineStr">
@@ -29402,7 +29402,7 @@
       </c>
       <c r="G576" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H576" s="2" t="inlineStr">
@@ -29502,7 +29502,7 @@
       </c>
       <c r="G578" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H578" s="2" t="inlineStr">
@@ -29552,7 +29552,7 @@
       </c>
       <c r="G579" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H579" s="4" t="inlineStr">
@@ -29652,7 +29652,7 @@
       </c>
       <c r="G581" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H581" s="4" t="inlineStr">
@@ -29702,7 +29702,7 @@
       </c>
       <c r="G582" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H582" s="2" t="inlineStr">
@@ -29810,7 +29810,7 @@
       </c>
       <c r="G584" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H584" s="2" t="inlineStr">
@@ -29860,7 +29860,7 @@
       </c>
       <c r="G585" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H585" s="4" t="inlineStr">
@@ -29960,7 +29960,7 @@
       </c>
       <c r="G587" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H587" s="4" t="inlineStr">
@@ -30010,7 +30010,7 @@
       </c>
       <c r="G588" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H588" s="2" t="inlineStr">
@@ -33560,7 +33560,7 @@
       </c>
       <c r="G659" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H659" s="4" t="inlineStr">
@@ -33610,7 +33610,7 @@
       </c>
       <c r="G660" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H660" s="2" t="inlineStr">
@@ -33710,7 +33710,7 @@
       </c>
       <c r="G662" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H662" s="2" t="inlineStr">
@@ -33760,7 +33760,7 @@
       </c>
       <c r="G663" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H663" s="4" t="inlineStr">
@@ -33860,7 +33860,7 @@
       </c>
       <c r="G665" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H665" s="4" t="inlineStr">
@@ -33910,7 +33910,7 @@
       </c>
       <c r="G666" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H666" s="2" t="inlineStr">
@@ -34010,7 +34010,7 @@
       </c>
       <c r="G668" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H668" s="2" t="inlineStr">
@@ -34060,7 +34060,7 @@
       </c>
       <c r="G669" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H669" s="4" t="inlineStr">
@@ -34160,7 +34160,7 @@
       </c>
       <c r="G671" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H671" s="4" t="inlineStr">
@@ -34210,7 +34210,7 @@
       </c>
       <c r="G672" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H672" s="2" t="inlineStr">
@@ -34310,7 +34310,7 @@
       </c>
       <c r="G674" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H674" s="2" t="inlineStr">
@@ -34360,7 +34360,7 @@
       </c>
       <c r="G675" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H675" s="4" t="inlineStr">
@@ -34460,7 +34460,7 @@
       </c>
       <c r="G677" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H677" s="4" t="inlineStr">
@@ -34510,7 +34510,7 @@
       </c>
       <c r="G678" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H678" s="2" t="inlineStr">
@@ -34610,7 +34610,7 @@
       </c>
       <c r="G680" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H680" s="2" t="inlineStr">
@@ -34660,7 +34660,7 @@
       </c>
       <c r="G681" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H681" s="4" t="inlineStr">
@@ -34760,7 +34760,7 @@
       </c>
       <c r="G683" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H683" s="4" t="inlineStr">
@@ -34818,7 +34818,7 @@
       </c>
       <c r="G684" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H684" s="2" t="inlineStr">
@@ -34918,7 +34918,7 @@
       </c>
       <c r="G686" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H686" s="2" t="inlineStr">
@@ -34968,7 +34968,7 @@
       </c>
       <c r="G687" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H687" s="4" t="inlineStr">
@@ -35068,7 +35068,7 @@
       </c>
       <c r="G689" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H689" s="4" t="inlineStr">
@@ -35118,7 +35118,7 @@
       </c>
       <c r="G690" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H690" s="2" t="inlineStr">
@@ -35218,7 +35218,7 @@
       </c>
       <c r="G692" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H692" s="2" t="inlineStr">
@@ -35268,7 +35268,7 @@
       </c>
       <c r="G693" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H693" s="4" t="inlineStr">
@@ -35368,7 +35368,7 @@
       </c>
       <c r="G695" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H695" s="4" t="inlineStr">
@@ -35418,7 +35418,7 @@
       </c>
       <c r="G696" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H696" s="2" t="inlineStr">
@@ -35518,7 +35518,7 @@
       </c>
       <c r="G698" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H698" s="2" t="inlineStr">
@@ -35568,7 +35568,7 @@
       </c>
       <c r="G699" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H699" s="4" t="inlineStr">
@@ -35668,7 +35668,7 @@
       </c>
       <c r="G701" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H701" s="4" t="inlineStr">
@@ -35718,7 +35718,7 @@
       </c>
       <c r="G702" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H702" s="2" t="inlineStr">
@@ -35818,7 +35818,7 @@
       </c>
       <c r="G704" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H704" s="2" t="inlineStr">
@@ -35868,7 +35868,7 @@
       </c>
       <c r="G705" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H705" s="4" t="inlineStr">
@@ -35968,7 +35968,7 @@
       </c>
       <c r="G707" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H707" s="4" t="inlineStr">
@@ -36018,7 +36018,7 @@
       </c>
       <c r="G708" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H708" s="2" t="inlineStr">
@@ -36126,7 +36126,7 @@
       </c>
       <c r="G710" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H710" s="2" t="inlineStr">
@@ -36176,7 +36176,7 @@
       </c>
       <c r="G711" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H711" s="4" t="inlineStr">
@@ -36276,7 +36276,7 @@
       </c>
       <c r="G713" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H713" s="4" t="inlineStr">
@@ -36326,7 +36326,7 @@
       </c>
       <c r="G714" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H714" s="2" t="inlineStr">
@@ -36426,7 +36426,7 @@
       </c>
       <c r="G716" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H716" s="2" t="inlineStr">
@@ -36476,7 +36476,7 @@
       </c>
       <c r="G717" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H717" s="4" t="inlineStr">
@@ -36576,7 +36576,7 @@
       </c>
       <c r="G719" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H719" s="4" t="inlineStr">
@@ -36626,7 +36626,7 @@
       </c>
       <c r="G720" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H720" s="2" t="inlineStr">
@@ -36726,7 +36726,7 @@
       </c>
       <c r="G722" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H722" s="2" t="inlineStr">
@@ -36776,7 +36776,7 @@
       </c>
       <c r="G723" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H723" s="4" t="inlineStr">
@@ -36876,7 +36876,7 @@
       </c>
       <c r="G725" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H725" s="4" t="inlineStr">
@@ -36926,7 +36926,7 @@
       </c>
       <c r="G726" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H726" s="2" t="inlineStr">
@@ -37026,7 +37026,7 @@
       </c>
       <c r="G728" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H728" s="2" t="inlineStr">
@@ -37076,7 +37076,7 @@
       </c>
       <c r="G729" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H729" s="4" t="inlineStr">
@@ -37176,7 +37176,7 @@
       </c>
       <c r="G731" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H731" s="4" t="inlineStr">
@@ -37226,7 +37226,7 @@
       </c>
       <c r="G732" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H732" s="2" t="inlineStr">
@@ -37334,7 +37334,7 @@
       </c>
       <c r="G734" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H734" s="2" t="inlineStr">
@@ -37384,7 +37384,7 @@
       </c>
       <c r="G735" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H735" s="4" t="inlineStr">
@@ -37484,7 +37484,7 @@
       </c>
       <c r="G737" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H737" s="4" t="inlineStr">
@@ -37534,7 +37534,7 @@
       </c>
       <c r="G738" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H738" s="2" t="inlineStr">
@@ -37634,7 +37634,7 @@
       </c>
       <c r="G740" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H740" s="2" t="inlineStr">
@@ -37684,7 +37684,7 @@
       </c>
       <c r="G741" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H741" s="4" t="inlineStr">
@@ -37784,7 +37784,7 @@
       </c>
       <c r="G743" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H743" s="4" t="inlineStr">
@@ -37834,7 +37834,7 @@
       </c>
       <c r="G744" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H744" s="2" t="inlineStr">
@@ -37934,7 +37934,7 @@
       </c>
       <c r="G746" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H746" s="2" t="inlineStr">
@@ -37984,7 +37984,7 @@
       </c>
       <c r="G747" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H747" s="4" t="inlineStr">
@@ -38084,7 +38084,7 @@
       </c>
       <c r="G749" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H749" s="4" t="inlineStr">
@@ -38134,7 +38134,7 @@
       </c>
       <c r="G750" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H750" s="2" t="inlineStr">
@@ -38234,7 +38234,7 @@
       </c>
       <c r="G752" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H752" s="2" t="inlineStr">
@@ -38284,7 +38284,7 @@
       </c>
       <c r="G753" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H753" s="4" t="inlineStr">
@@ -38384,7 +38384,7 @@
       </c>
       <c r="G755" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H755" s="4" t="inlineStr">
@@ -38434,7 +38434,7 @@
       </c>
       <c r="G756" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H756" s="2" t="inlineStr">
@@ -38534,7 +38534,7 @@
       </c>
       <c r="G758" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H758" s="2" t="inlineStr">
@@ -38592,7 +38592,7 @@
       </c>
       <c r="G759" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H759" s="4" t="inlineStr">
@@ -38692,7 +38692,7 @@
       </c>
       <c r="G761" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H761" s="4" t="inlineStr">
@@ -38742,7 +38742,7 @@
       </c>
       <c r="G762" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H762" s="2" t="inlineStr">
@@ -38842,7 +38842,7 @@
       </c>
       <c r="G764" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H764" s="2" t="inlineStr">
@@ -38892,7 +38892,7 @@
       </c>
       <c r="G765" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H765" s="4" t="inlineStr">
@@ -38992,7 +38992,7 @@
       </c>
       <c r="G767" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H767" s="4" t="inlineStr">
@@ -39042,7 +39042,7 @@
       </c>
       <c r="G768" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H768" s="2" t="inlineStr">
@@ -39142,7 +39142,7 @@
       </c>
       <c r="G770" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H770" s="2" t="inlineStr">
@@ -39192,7 +39192,7 @@
       </c>
       <c r="G771" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H771" s="4" t="inlineStr">
@@ -39292,7 +39292,7 @@
       </c>
       <c r="G773" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H773" s="4" t="inlineStr">
@@ -39342,7 +39342,7 @@
       </c>
       <c r="G774" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H774" s="2" t="inlineStr">
@@ -39442,7 +39442,7 @@
       </c>
       <c r="G776" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H776" s="2" t="inlineStr">
@@ -39492,7 +39492,7 @@
       </c>
       <c r="G777" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H777" s="4" t="inlineStr">
@@ -39592,7 +39592,7 @@
       </c>
       <c r="G779" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H779" s="4" t="inlineStr">
@@ -39642,7 +39642,7 @@
       </c>
       <c r="G780" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H780" s="2" t="inlineStr">
@@ -39742,7 +39742,7 @@
       </c>
       <c r="G782" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H782" s="2" t="inlineStr">
@@ -39792,7 +39792,7 @@
       </c>
       <c r="G783" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H783" s="4" t="inlineStr">
@@ -39900,7 +39900,7 @@
       </c>
       <c r="G785" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H785" s="4" t="inlineStr">
@@ -39950,7 +39950,7 @@
       </c>
       <c r="G786" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H786" s="2" t="inlineStr">
@@ -40050,7 +40050,7 @@
       </c>
       <c r="G788" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H788" s="2" t="inlineStr">
@@ -40100,7 +40100,7 @@
       </c>
       <c r="G789" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H789" s="4" t="inlineStr">
@@ -43702,7 +43702,7 @@
       </c>
       <c r="G860" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H860" s="2" t="inlineStr">
@@ -43752,7 +43752,7 @@
       </c>
       <c r="G861" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H861" s="4" t="inlineStr">
@@ -43852,7 +43852,7 @@
       </c>
       <c r="G863" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H863" s="4" t="inlineStr">
@@ -43902,7 +43902,7 @@
       </c>
       <c r="G864" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H864" s="2" t="inlineStr">
@@ -44002,7 +44002,7 @@
       </c>
       <c r="G866" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H866" s="2" t="inlineStr">
@@ -44052,7 +44052,7 @@
       </c>
       <c r="G867" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H867" s="4" t="inlineStr">
@@ -44152,7 +44152,7 @@
       </c>
       <c r="G869" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H869" s="4" t="inlineStr">
@@ -44202,7 +44202,7 @@
       </c>
       <c r="G870" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H870" s="2" t="inlineStr">
@@ -44302,7 +44302,7 @@
       </c>
       <c r="G872" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H872" s="2" t="inlineStr">
@@ -44352,7 +44352,7 @@
       </c>
       <c r="G873" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H873" s="4" t="inlineStr">
@@ -44452,7 +44452,7 @@
       </c>
       <c r="G875" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H875" s="4" t="inlineStr">
@@ -44502,7 +44502,7 @@
       </c>
       <c r="G876" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H876" s="2" t="inlineStr">
@@ -44602,7 +44602,7 @@
       </c>
       <c r="G878" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H878" s="2" t="inlineStr">
@@ -44652,7 +44652,7 @@
       </c>
       <c r="G879" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H879" s="4" t="inlineStr">
@@ -44752,7 +44752,7 @@
       </c>
       <c r="G881" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H881" s="4" t="inlineStr">
@@ -44802,7 +44802,7 @@
       </c>
       <c r="G882" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H882" s="2" t="inlineStr">
@@ -44902,7 +44902,7 @@
       </c>
       <c r="G884" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H884" s="2" t="inlineStr">
@@ -44960,7 +44960,7 @@
       </c>
       <c r="G885" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H885" s="4" t="inlineStr">
@@ -45060,7 +45060,7 @@
       </c>
       <c r="G887" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H887" s="4" t="inlineStr">
@@ -45110,7 +45110,7 @@
       </c>
       <c r="G888" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H888" s="2" t="inlineStr">
@@ -45210,7 +45210,7 @@
       </c>
       <c r="G890" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H890" s="2" t="inlineStr">
@@ -45260,7 +45260,7 @@
       </c>
       <c r="G891" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H891" s="4" t="inlineStr">
@@ -45360,7 +45360,7 @@
       </c>
       <c r="G893" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H893" s="4" t="inlineStr">
@@ -45410,7 +45410,7 @@
       </c>
       <c r="G894" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H894" s="2" t="inlineStr">
@@ -45510,7 +45510,7 @@
       </c>
       <c r="G896" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H896" s="2" t="inlineStr">
@@ -45560,7 +45560,7 @@
       </c>
       <c r="G897" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H897" s="4" t="inlineStr">
@@ -45660,7 +45660,7 @@
       </c>
       <c r="G899" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H899" s="4" t="inlineStr">
@@ -45710,7 +45710,7 @@
       </c>
       <c r="G900" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H900" s="2" t="inlineStr">
@@ -45810,7 +45810,7 @@
       </c>
       <c r="G902" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H902" s="2" t="inlineStr">
@@ -45860,7 +45860,7 @@
       </c>
       <c r="G903" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H903" s="4" t="inlineStr">
@@ -45960,7 +45960,7 @@
       </c>
       <c r="G905" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H905" s="4" t="inlineStr">
@@ -46010,7 +46010,7 @@
       </c>
       <c r="G906" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H906" s="2" t="inlineStr">
@@ -46110,7 +46110,7 @@
       </c>
       <c r="G908" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H908" s="2" t="inlineStr">
@@ -46160,7 +46160,7 @@
       </c>
       <c r="G909" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H909" s="4" t="inlineStr">
@@ -46268,7 +46268,7 @@
       </c>
       <c r="G911" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H911" s="4" t="inlineStr">
@@ -46318,7 +46318,7 @@
       </c>
       <c r="G912" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H912" s="2" t="inlineStr">
@@ -46418,7 +46418,7 @@
       </c>
       <c r="G914" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H914" s="2" t="inlineStr">
@@ -46468,7 +46468,7 @@
       </c>
       <c r="G915" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H915" s="4" t="inlineStr">
@@ -46568,7 +46568,7 @@
       </c>
       <c r="G917" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H917" s="4" t="inlineStr">
@@ -46618,7 +46618,7 @@
       </c>
       <c r="G918" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H918" s="2" t="inlineStr">
@@ -46718,7 +46718,7 @@
       </c>
       <c r="G920" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H920" s="2" t="inlineStr">
@@ -46768,7 +46768,7 @@
       </c>
       <c r="G921" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H921" s="4" t="inlineStr">
@@ -46868,7 +46868,7 @@
       </c>
       <c r="G923" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H923" s="4" t="inlineStr">
@@ -46918,7 +46918,7 @@
       </c>
       <c r="G924" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H924" s="2" t="inlineStr">
@@ -47018,7 +47018,7 @@
       </c>
       <c r="G926" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H926" s="2" t="inlineStr">
@@ -47068,7 +47068,7 @@
       </c>
       <c r="G927" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H927" s="4" t="inlineStr">
@@ -47168,7 +47168,7 @@
       </c>
       <c r="G929" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H929" s="4" t="inlineStr">
@@ -47218,7 +47218,7 @@
       </c>
       <c r="G930" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H930" s="2" t="inlineStr">
@@ -47318,7 +47318,7 @@
       </c>
       <c r="G932" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H932" s="2" t="inlineStr">
@@ -47368,7 +47368,7 @@
       </c>
       <c r="G933" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H933" s="4" t="inlineStr">
@@ -47476,7 +47476,7 @@
       </c>
       <c r="G935" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H935" s="4" t="inlineStr">
@@ -47526,7 +47526,7 @@
       </c>
       <c r="G936" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H936" s="2" t="inlineStr">
@@ -47626,7 +47626,7 @@
       </c>
       <c r="G938" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H938" s="2" t="inlineStr">
@@ -47676,7 +47676,7 @@
       </c>
       <c r="G939" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H939" s="4" t="inlineStr">
@@ -47776,7 +47776,7 @@
       </c>
       <c r="G941" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H941" s="4" t="inlineStr">
@@ -47826,7 +47826,7 @@
       </c>
       <c r="G942" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H942" s="2" t="inlineStr">
@@ -47926,7 +47926,7 @@
       </c>
       <c r="G944" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H944" s="2" t="inlineStr">
@@ -47976,7 +47976,7 @@
       </c>
       <c r="G945" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H945" s="4" t="inlineStr">
@@ -48076,7 +48076,7 @@
       </c>
       <c r="G947" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H947" s="4" t="inlineStr">
@@ -48126,7 +48126,7 @@
       </c>
       <c r="G948" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H948" s="2" t="inlineStr">
@@ -48226,7 +48226,7 @@
       </c>
       <c r="G950" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H950" s="2" t="inlineStr">
@@ -48276,7 +48276,7 @@
       </c>
       <c r="G951" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H951" s="4" t="inlineStr">
@@ -48376,7 +48376,7 @@
       </c>
       <c r="G953" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H953" s="4" t="inlineStr">
@@ -48426,7 +48426,7 @@
       </c>
       <c r="G954" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H954" s="2" t="inlineStr">
@@ -48526,7 +48526,7 @@
       </c>
       <c r="G956" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H956" s="2" t="inlineStr">
@@ -48576,7 +48576,7 @@
       </c>
       <c r="G957" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H957" s="4" t="inlineStr">
@@ -48676,7 +48676,7 @@
       </c>
       <c r="G959" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H959" s="4" t="inlineStr">
@@ -48734,7 +48734,7 @@
       </c>
       <c r="G960" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H960" s="2" t="inlineStr">
@@ -48834,7 +48834,7 @@
       </c>
       <c r="G962" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H962" s="2" t="inlineStr">
@@ -48884,7 +48884,7 @@
       </c>
       <c r="G963" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H963" s="4" t="inlineStr">
@@ -48984,7 +48984,7 @@
       </c>
       <c r="G965" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H965" s="4" t="inlineStr">
@@ -49034,7 +49034,7 @@
       </c>
       <c r="G966" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H966" s="2" t="inlineStr">
@@ -49134,7 +49134,7 @@
       </c>
       <c r="G968" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H968" s="2" t="inlineStr">
@@ -49184,7 +49184,7 @@
       </c>
       <c r="G969" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H969" s="4" t="inlineStr">
@@ -49284,7 +49284,7 @@
       </c>
       <c r="G971" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H971" s="4" t="inlineStr">
@@ -49334,7 +49334,7 @@
       </c>
       <c r="G972" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H972" s="2" t="inlineStr">
@@ -49434,7 +49434,7 @@
       </c>
       <c r="G974" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H974" s="2" t="inlineStr">
@@ -49484,7 +49484,7 @@
       </c>
       <c r="G975" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H975" s="4" t="inlineStr">
@@ -49584,7 +49584,7 @@
       </c>
       <c r="G977" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H977" s="4" t="inlineStr">
@@ -49634,7 +49634,7 @@
       </c>
       <c r="G978" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H978" s="2" t="inlineStr">
@@ -49734,7 +49734,7 @@
       </c>
       <c r="G980" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H980" s="2" t="inlineStr">
@@ -49784,7 +49784,7 @@
       </c>
       <c r="G981" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H981" s="4" t="inlineStr">
@@ -49884,7 +49884,7 @@
       </c>
       <c r="G983" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H983" s="4" t="inlineStr">
@@ -49934,7 +49934,7 @@
       </c>
       <c r="G984" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H984" s="2" t="inlineStr">
@@ -50042,7 +50042,7 @@
       </c>
       <c r="G986" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H986" s="2" t="inlineStr">
@@ -50092,7 +50092,7 @@
       </c>
       <c r="G987" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H987" s="4" t="inlineStr">
@@ -50192,7 +50192,7 @@
       </c>
       <c r="G989" s="4" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>CCE工作负载</t>
         </is>
       </c>
       <c r="H989" s="4" t="inlineStr">
@@ -50242,7 +50242,7 @@
       </c>
       <c r="G990" s="2" t="inlineStr">
         <is>
-          <t>CCE_Deployment</t>
+          <t>K8s集群</t>
         </is>
       </c>
       <c r="H990" s="2" t="inlineStr">

</xml_diff>